<commit_message>
Add SQL practice sets for Constraints & DML at various difficulty levels
- Created 100-question practice set for CRAZY level focusing on advanced DML patterns including idempotent writes, CDC, and bulk loading.
- Created 100-question practice set for EASY level covering basic constraints, keys, and DML operations.
- Created 100-question practice set for HARD level emphasizing UPSERT, MERGE, and writeable CTEs.
- Created 100-question practice set for MEDIUM level exploring complex constraints, bulk DML, and transactional CRUD patterns.
</commit_message>
<xml_diff>
--- a/batch_notes/28/batch_28.xlsx
+++ b/batch_notes/28/batch_28.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10804"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/shira_2/__work__/acciojob/modules/sql/postgresql/batch_notes/28/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0D360A-A820-BE46-8D8F-4D825F974A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838724BE-F9F5-1A41-8C1E-35F86F41396D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-2480" windowWidth="38400" windowHeight="21600" xr2:uid="{C88571CB-2605-694D-B9DF-E4D6E422F2C7}"/>
+    <workbookView xWindow="-38400" yWindow="-2480" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{C88571CB-2605-694D-B9DF-E4D6E422F2C7}"/>
   </bookViews>
   <sheets>
     <sheet name="01" sheetId="1" r:id="rId1"/>
+    <sheet name="02" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
   <si>
     <t>Warehouse</t>
   </si>
@@ -162,6 +163,120 @@
   </si>
   <si>
     <t>loyalty</t>
+  </si>
+  <si>
+    <t>Steps</t>
+  </si>
+  <si>
+    <t>open git repo</t>
+  </si>
+  <si>
+    <t>https://github.com/starlordali4444/postgresql.git</t>
+  </si>
+  <si>
+    <t>open vs code</t>
+  </si>
+  <si>
+    <t>in vs code click on open folder</t>
+  </si>
+  <si>
+    <t>create sql folder in any location except ondrive</t>
+  </si>
+  <si>
+    <t>open terminal in vs code</t>
+  </si>
+  <si>
+    <t>enter command =&gt; git clone https://github.com/starlordali4444/postgresql.git</t>
+  </si>
+  <si>
+    <t>wait for cloning</t>
+  </si>
+  <si>
+    <t>once done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enter in terminal =&gt; cd postgre </t>
+  </si>
+  <si>
+    <t>press tab</t>
+  </si>
+  <si>
+    <t>psql -U postgres -d postgres -f datasets\v3\sql\setup_accio_retailmart.sql</t>
+  </si>
+  <si>
+    <t>once its completed keep pressing enter to get all the tables</t>
+  </si>
+  <si>
+    <t>then go to pgadmin 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">right click on databases </t>
+  </si>
+  <si>
+    <t>click refresh</t>
+  </si>
+  <si>
+    <t>you will see accio_retailmart_ database</t>
+  </si>
+  <si>
+    <t>click on the above database to connect</t>
+  </si>
+  <si>
+    <t>right click on the above database then click on properties</t>
+  </si>
+  <si>
+    <t>add 28 in the of database name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">click ok </t>
+  </si>
+  <si>
+    <t xml:space="preserve">we are done </t>
+  </si>
+  <si>
+    <t>Books</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>Borrowing/Returning</t>
+  </si>
+  <si>
+    <t>Schemas</t>
+  </si>
+  <si>
+    <t>Column2</t>
+  </si>
+  <si>
+    <t>Column3</t>
+  </si>
+  <si>
+    <t>Column4</t>
+  </si>
+  <si>
+    <t>Column5</t>
+  </si>
+  <si>
+    <t>Student_id</t>
+  </si>
+  <si>
+    <t>Ali</t>
+  </si>
+  <si>
+    <t>accio_28</t>
+  </si>
+  <si>
+    <t>shop</t>
+  </si>
+  <si>
+    <t>people</t>
+  </si>
+  <si>
+    <t>transaction</t>
+  </si>
+  <si>
+    <t>table</t>
   </si>
 </sst>
 </file>
@@ -191,7 +306,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -199,13 +314,102 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -238,8 +442,8 @@
       <xdr:row>12</xdr:row>
       <xdr:rowOff>139920</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="2" name="Ink 1">
@@ -258,7 +462,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="2" name="Ink 1">
@@ -303,8 +507,8 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>34720</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="3" name="Ink 2">
@@ -323,7 +527,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="3" name="Ink 2">
@@ -368,8 +572,8 @@
       <xdr:row>12</xdr:row>
       <xdr:rowOff>167640</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="4" name="Ink 3">
@@ -388,7 +592,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="4" name="Ink 3">
@@ -418,6 +622,55 @@
         </xdr:pic>
       </mc:Fallback>
     </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>163133</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{050000E6-E3C0-4421-00E1-256041CF8A4B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1651000" y="3048000"/>
+          <a:ext cx="7772400" cy="3617533"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -502,6 +755,20 @@
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">4094 200 24575,'-5'-5'0,"-4"1"0,-19-9 0,-30-6 0,-33-4 0,32 11 0,-4 3 0,-9 1 0,2 2 0,-23 2 0,37 2 0,4 1 0,1 1 0,-37-8 0,-21-3 0,21 6 0,-6 1 0,-8-1-646,14 1 1,-8-1 0,-3 1 0,0-1 0,3 2 645,9 0 0,3 1 0,0 0 0,-2 0 0,-3 1 0,-1 0 0,-4 1 0,-2 0 0,0 1 0,2-1 0,5 0 0,2 0 0,3 0 0,3 0 0,-1 0 0,0 0-360,-5 0 1,-2-1 0,0 0 0,4 0 0,4 0 359,-20 0 0,7 0 0,9 0 0,0-1 0,16-1 0,16-2 0,16 2 0,15 1 2889,-6-3-2889,15 4 2133,9-1-2133,17 6 0,16-3 0,1 3 0,-6-4 0,-13 0 0</inkml:trace>
 </inkml:ink>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3CF7AC3A-5F42-EF48-A52B-FC82AB433DE0}" name="Table1" displayName="Table1" ref="I67:M79" totalsRowShown="0">
+  <autoFilter ref="I67:M79" xr:uid="{3CF7AC3A-5F42-EF48-A52B-FC82AB433DE0}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{6D6DB51D-16FE-5A42-966B-22D3B6FB2EEC}" name="Student_id"/>
+    <tableColumn id="2" xr3:uid="{F1607987-4049-D149-AB53-6369820C76A7}" name="Column2"/>
+    <tableColumn id="3" xr3:uid="{86AE4211-B9CF-1240-80C4-1BAD3EAB3AEF}" name="Column3"/>
+    <tableColumn id="4" xr3:uid="{61DFAD3D-3AB7-114F-A2F9-1CC2946365B4}" name="Column4"/>
+    <tableColumn id="5" xr3:uid="{1192BE98-3F1F-5849-AEA8-B2AF03CE16F9}" name="Column5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1061,4 +1328,463 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C30BBE9F-6251-054D-8156-7574F8262F96}">
+  <dimension ref="B2:M88"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B34">
+        <v>13</v>
+      </c>
+      <c r="C34" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B35">
+        <v>14</v>
+      </c>
+      <c r="C35" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B36">
+        <v>15</v>
+      </c>
+      <c r="C36" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B37">
+        <v>16</v>
+      </c>
+      <c r="C37" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B38">
+        <v>17</v>
+      </c>
+      <c r="C38" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B39">
+        <v>18</v>
+      </c>
+      <c r="C39" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B40">
+        <v>19</v>
+      </c>
+      <c r="C40" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B41">
+        <v>20</v>
+      </c>
+      <c r="C41" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B42">
+        <v>21</v>
+      </c>
+      <c r="C42" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="51" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D51" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>67</v>
+      </c>
+      <c r="D52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F52" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="53" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B53" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C53" s="4"/>
+      <c r="D53" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E53" s="4"/>
+      <c r="F53" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G53" s="4"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="3"/>
+      <c r="K53" s="3"/>
+      <c r="L53" s="4"/>
+    </row>
+    <row r="54" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B54" s="5"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="7"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="6"/>
+      <c r="K54" s="6"/>
+      <c r="L54" s="7"/>
+    </row>
+    <row r="55" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B55" s="5"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="7"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
+      <c r="L55" s="7"/>
+    </row>
+    <row r="56" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B56" s="5"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="7"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="6"/>
+      <c r="K56" s="6"/>
+      <c r="L56" s="7"/>
+    </row>
+    <row r="57" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B57" s="5"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="7"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="6"/>
+      <c r="K57" s="6"/>
+      <c r="L57" s="7"/>
+    </row>
+    <row r="58" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B58" s="5"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="7"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="6"/>
+      <c r="K58" s="6"/>
+      <c r="L58" s="7"/>
+    </row>
+    <row r="59" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B59" s="5"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="6"/>
+      <c r="G59" s="7"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="6"/>
+      <c r="K59" s="6"/>
+      <c r="L59" s="7"/>
+    </row>
+    <row r="60" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B60" s="5"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="7"/>
+      <c r="I60" s="5"/>
+      <c r="J60" s="6"/>
+      <c r="K60" s="6"/>
+      <c r="L60" s="7"/>
+    </row>
+    <row r="61" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B61" s="5"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="7"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="6"/>
+      <c r="K61" s="6"/>
+      <c r="L61" s="7"/>
+    </row>
+    <row r="62" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B62" s="5"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="6"/>
+      <c r="G62" s="7"/>
+      <c r="I62" s="5"/>
+      <c r="J62" s="6"/>
+      <c r="K62" s="6"/>
+      <c r="L62" s="7"/>
+    </row>
+    <row r="63" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B63" s="5"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="7"/>
+      <c r="I63" s="8"/>
+      <c r="J63" s="9"/>
+      <c r="K63" s="9"/>
+      <c r="L63" s="10"/>
+    </row>
+    <row r="64" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B64" s="5"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="7"/>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B65" s="5"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="6"/>
+      <c r="G65" s="7"/>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B66" s="5"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="7"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="7"/>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B67" s="5"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="7"/>
+      <c r="I67" t="s">
+        <v>72</v>
+      </c>
+      <c r="J67" t="s">
+        <v>68</v>
+      </c>
+      <c r="K67" t="s">
+        <v>69</v>
+      </c>
+      <c r="L67" t="s">
+        <v>70</v>
+      </c>
+      <c r="M67" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="68" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B68" s="5"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="7"/>
+      <c r="I68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B69" s="5"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="7"/>
+      <c r="I69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="8"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="10"/>
+      <c r="F70" s="9"/>
+      <c r="G70" s="10"/>
+      <c r="I70">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="I71" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="83" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C83" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="84" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D84" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="85" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E85" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="86" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E86" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="87" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D87" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="88" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D88" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove documentation and master runner script from RetailMart analytics project
- Deleted README.md file from the documentation directory, which contained project overview, setup instructions, and analytics details.
- Removed day_27_28_29.xlsx, an Excel file from the documentation directory.
- Eliminated run_all.sql, the master runner script for building the entire analytics layer.
</commit_message>
<xml_diff>
--- a/batch_notes/28/batch_28.xlsx
+++ b/batch_notes/28/batch_28.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/shira_2/__work__/acciojob/modules/sql/postgresql/batch_notes/28/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33391F5C-9BF9-4040-9E83-25B3D02CD98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C6F2891-C59B-CB4E-B1F4-9273FA0399E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-2480" windowWidth="38400" windowHeight="21600" activeTab="9" xr2:uid="{C88571CB-2605-694D-B9DF-E4D6E422F2C7}"/>
+    <workbookView xWindow="-38400" yWindow="-2480" windowWidth="38400" windowHeight="21600" activeTab="10" xr2:uid="{C88571CB-2605-694D-B9DF-E4D6E422F2C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Intro to SQL" sheetId="1" r:id="rId1"/>
@@ -23,12 +23,13 @@
     <sheet name="Aggregate Functions &amp; Group By" sheetId="8" r:id="rId8"/>
     <sheet name="Join Part 1 &amp; 2" sheetId="9" r:id="rId9"/>
     <sheet name="Self Join" sheetId="10" r:id="rId10"/>
+    <sheet name="Subquery" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId11"/>
-    <pivotCache cacheId="1" r:id="rId12"/>
-    <pivotCache cacheId="2" r:id="rId13"/>
+    <pivotCache cacheId="0" r:id="rId12"/>
+    <pivotCache cacheId="1" r:id="rId13"/>
+    <pivotCache cacheId="2" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -75,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="773">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="785">
   <si>
     <t>Warehouse</t>
   </si>
@@ -2424,6 +2425,42 @@
   </si>
   <si>
     <t>Food Taste</t>
+  </si>
+  <si>
+    <t>Complete Value</t>
+  </si>
+  <si>
+    <t>part of the string</t>
+  </si>
+  <si>
+    <t>Outer</t>
+  </si>
+  <si>
+    <t>Execute Inner</t>
+  </si>
+  <si>
+    <t>Output of inner will be used by Outer Query</t>
+  </si>
+  <si>
+    <t>Quter Query will be executed and we get the result</t>
+  </si>
+  <si>
+    <t>OutPut</t>
+  </si>
+  <si>
+    <t>Multi Row</t>
+  </si>
+  <si>
+    <t>Derived Table</t>
+  </si>
+  <si>
+    <t>If you have one ticket for concert how many people can go</t>
+  </si>
+  <si>
+    <t>If we have group ticket where I can have 5 people</t>
+  </si>
+  <si>
+    <t>IN | NOT IN</t>
   </si>
 </sst>
 </file>
@@ -2765,7 +2802,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -2862,6 +2899,10 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2937,10 +2978,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6727,6 +6773,579 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>368300</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>15373</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4340FC3D-70B7-814D-D2B5-2E6FDE2B8C7D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="203200"/>
+          <a:ext cx="7772400" cy="4079373"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>787400</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>387350</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Frame 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6030AA0-01A3-3635-A3B3-98A0E0851DF4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="787400" y="215900"/>
+          <a:ext cx="7829550" cy="4051300"/>
+        </a:xfrm>
+        <a:prstGeom prst="frame">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 2312"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Frame 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7779D85D-75B3-8E46-BE95-5CC7A405D78D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1244600" y="2673350"/>
+          <a:ext cx="7213600" cy="1454150"/>
+        </a:xfrm>
+        <a:prstGeom prst="frame">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 4432"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent2">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>660400</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Frame 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E77E77FD-619A-594A-AEFA-457E8F5C7B53}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="850900" y="4489450"/>
+          <a:ext cx="5588000" cy="2089150"/>
+        </a:xfrm>
+        <a:prstGeom prst="frame">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 2312"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>565150</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>482600</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Frame 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EAE593D4-3674-7B42-8586-B9F50C2B299A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1390650" y="4972050"/>
+          <a:ext cx="4870450" cy="1492250"/>
+        </a:xfrm>
+        <a:prstGeom prst="frame">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 4432"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent2">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>617620</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>112760</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>504560</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>108480</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="7" name="Ink 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2EBAFF0E-BA5B-4EAF-5C13-2C2B3E925D5D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="6396120" y="4583160"/>
+            <a:ext cx="712440" cy="402120"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="7" name="Ink 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2EBAFF0E-BA5B-4EAF-5C13-2C2B3E925D5D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="6391800" y="4578840"/>
+              <a:ext cx="721080" cy="410760"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>769920</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>160320</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>399460</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>141640</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="8" name="Ink 7">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4D085D25-E51C-3274-5C47-3437FEA3AD30}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="5722920" y="5037120"/>
+            <a:ext cx="455040" cy="387720"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="8" name="Ink 7">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4D085D25-E51C-3274-5C47-3437FEA3AD30}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="5718600" y="5032800"/>
+              <a:ext cx="463680" cy="396360"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>448440</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>60840</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>713360</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>129120</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="21" name="Ink 20">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E1F5FC4-8EB9-4AE1-59E7-BB336ED1C60E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="5401440" y="5547240"/>
+            <a:ext cx="1915920" cy="677880"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="21" name="Ink 20">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E1F5FC4-8EB9-4AE1-59E7-BB336ED1C60E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="5397120" y="5542920"/>
+              <a:ext cx="1924560" cy="686520"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>52580</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>152320</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>699860</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>92600</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="22" name="Ink 21">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{761913C4-06C0-74FC-206B-41DD2344C1FD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7456680" y="13588920"/>
+            <a:ext cx="647280" cy="346680"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="22" name="Ink 21">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{761913C4-06C0-74FC-206B-41DD2344C1FD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7452360" y="13584600"/>
+              <a:ext cx="655920" cy="355320"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
@@ -7533,6 +8152,124 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">4730 484,'-41'1,"1"5,13 16,-18 14,-4 3,5-4,14-8,17-17,1 7,3-5,1-1,-20 26,0-7,-11 16,14-15,5 3,7-5,-7 5,1 2,-23 22,8 15,-8 4,20-10,1 2,-11 21,2 2,-1 2,13-35,-1-4,-7 10,1-4,4 15,0-36,11-10,-1-6,5-10,-5 14,7-9,-1-2,5-3,-3-2,3 10,-2-7,4 7,8 21,0 30,3-5,-7-1,-2-38,0-2,3-4,5 20,-2-24,0 23,-7-31,2 14,-1-13,14 51,9 20,-15-33,1 0,18 43,-16-46,1-17,-8-15,-1-8,3 7,5-3,0 4,-1-5,-2-7,14 45,-12-13,20 50,-26-47,5-3,-9-23,-4 15,5 6,-4 9,4-13,-5-11,-17 69,14-2,2 7,-8-9,1 1,6 17,4-14,0-35,15-12,-6-34,11 13,-12-16,1 4,10-4,0 12,8 15,-2 1,-11 13,0-19,-9-5,-2-6,2-4,2 5,2 7,-2-8,4 4,-1-12,6-1,-3-2,4-6,-3 3,-3-2,17 2,-18 0,14 2,-14 3,6 3,-7 2,3 1,2 2,14 7,-6-7,4 3,-23-11,-5 19,5 52,5 7,2-4,1-2,3-7,-2 7,-19-75,-1-2,-23-7,16 6,-19-4,6 13,-24 0,-33 13,7-5,-6 0,7 1,2-1,1 1,4-2,-17 5,61-13,5-2,5 2,0-1,-23 7,15-5,-24 5,18-9,-12 0,8-4,4 0,3 0,13 0,-26 0,-12 8,0-2,2 6,24-5,11-4,1-1,-17-2,15 0,-12 0,16 0,-4 0,-4-5,-34-7,23 4,-30-10,4 1,-9-1,-30-4,-6-1,9 0,-1 0,19 8,-3 2,13 1,-13-3,8-1,2 1,-9 2,21 6,1 0,-22 0,15-5,39 2,-50-36,-4 5,18 5,2 0,-12-1,24 3,27 19,-8-9,-18-17,-11 5,-16-22,3 22,9-3,2 0,29 24,-8-21,19 23,-41-53,17 33,-5-14,-2-2,-16-4,20 11,1 0,-7 0,10 3,15 14,-10-29,-4-5,-15-13,-6-7,19 22,1 1,-16-17,0-1,7 10,3 4,10 11,0 1,-3 0,2 1,-13-29,27 43,8 3,8 18,0 0,1-18,0-32,0-14,9 3,2-2,-3 23,0-1,4-25,2 0,4 19,-1 2,-3 1,2-1,11-10,3 2,-7 17,2 0,9-14,2-2,2 1,0 3,-7 16,-1 0,2-6,0 0,18-26,-19 31,2-1,0 3,0-1,5-9,1 2,25-23,-4-5,-16 30,-5 1,-11 11,13-7,0 1,19-5,-1 4,-16 14,4-2,19-17,0-1,-12 16,1 1,27-20,-2 4,4 9,-26 18,0 1,11-6,6 1,-14-5,3-4,-7 6,0 0,7-5,-1 1,-8 5,-1 4,38 0,-3 2,12 12,-47 7,3 3,34 6,8 1,0-6,5 1,-3 6,5 3,-9-3,-10-5,-7-1,4 4,-15 2,-35-2,-4 3,-7 4,6 5,-7-5,2 2,-9-8,3 1,-59 22,-4-3,-8 2,-13 5,-10 4,10-7,-10 4,-1 2,4-1,-9 10,5 2,-3-2,15-10,-4 0,3 0,4-1,3 4,4-1,2-1,-22 14,3-3,19-14,1 0,-6 10,4-2,-3 4,33-15,8-14,-21 41,17-21,-7 16,31-28,4-21,62 1,-12-11,8-6,8-4,9-4,3-7,-6-6,4-6,1-3,-3-1,-3 4,-1-2,-1-1,-2-3,1-6,0-5,-4 1,-5 4,-3 6,-5 2,-7 3,-3-6,-7 6,5 3,-40 27,-58 25,-53 29,-2 3,34-15,-1 2,-4 2,-5 4,15-7,-6 3,-2 3,-3 0,0 2,2 0,2 1,-10 5,1 2,1 0,2 1,2 0,4 1,-1 2,4 0,2 0,3 2,3 1,-12 13,3 4,5-3,10-7,-4 6,13-6,13-2,16-15,23-39,5-2,60-33,32-24,-30 19,4-3,12-11,-23 11,9-7,7-5,4-4,3-2,0-1,-3 1,-4 3,-6 3,5-4,-5 2,-3 1,-1 0,2-1,3-3,5-3,5-4,4-2,-2 0,-4 2,-9 3,-10 7,5-14,-13 6,-14 13,-8 10,-90 101,13-9,-9 12,-6 7,4-10,-5 5,-3 4,-3 3,-1 4,17-18,-2 3,-1 3,-1 2,0 0,1 0,2-2,2-3,-6 9,3-2,1-1,1-1,1-1,1 1,-10 10,-1 3,3-2,6-6,13-12,-1 12,24-21,29-36,23-49,13-25,-1 10,5-4,4-5,3-8,3-7,2-2,1 0,2 1,1 0,2-1,3-4,-12 12,3-5,2-2,-2 2,-3 3,-6 8,8-9,-6 7,0 0,20-21,1-1,-39 46,-62 74,-13 22,-12 20,-1 3,15-20,0 2,-1 1,-1 4,0-1,-3 5,0 2,2-4,3-6,-2 8,3-6,6-7,0 6,15-29,14-40,39-75,-11 32,4-5,4-7,4-5,-3 3,0 0,-3 4,3-3,-11 26,-44 105,-3-15,-5 12,-5 5,-2 4,-4 5,-2 5,-1 1,3-5,-1 5,0 1,0-3,2-6,0-5,2-5,1-3,2-2,-11 21,3-3,27-44,41-67,13-24,2-15,4-13,-6 15,6-8,1-4,-3 3,-5 3,-1-1,-1 1,-1 2,7-13,-2 3,-3 7,2-9,-14 34,-27 51,-21 48,-21 37,-2 0,6-11,-1 0,-6 7,2-5,-6 9,-3 2,3-4,6-12,4-7,5-8,-1-2,-11 16,-1-1,24-43,28-47,28-45,9-18,-8 1,1-5,2 9,4-4,-7 7,-3-8,-14 34,-33 112,-17 48,12-47,-2 2,-2 8,1-4,-1 10,-1 2,1-2,4-9,0 7,4-8,2-6,-3 12,13-34,43-93,-10-4,2-12,2-11,3-11,-1 8,5 2,-3 6,-5-11,-9 32,-15 74,-17 52,-7 17,6-24,1 0,-6 22,5-11,10-34,19-70,12-33,7-16,-5 10,2-4,0 2,11-23,-3 4,-2 8,-8 16,-21 40,-24 79,-12 17,-12 11,2-13,62-123,15-30,-15 21,2-2,4-1,4-4,-4 10,16-11,-50 110,-11 33,-1 10,-3 9,0-6,-2 6,0-8,-1-3,0-15,-4-11,27-122,9-39,-3 11,1-1,3-7,0 8,3 5,-11 62,-6 24,26 22,16-5,4 2,18 17,-16-18,-6-5,-26-12,-10-26,-4-9,8-26,-7 22,2-3,-6 31,1 3</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink36.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-08-29T14:41:22.085"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1979 8 24575,'-2'-5'0,"-4"3"0,-11 7 0,1-2 0,-16 8 0,-5-4 0,-18 7 0,-24 5 0,11 1 0,-16 6 0,48-9 0,-2-1 0,28-9 0,-3 4 0,-23 3 0,1 2 0,-45 12 0,33-8 0,-21 10 0,17-5 0,10-2 0,6-5 0,16-8 0,12-10 0,0 0 0,-2 0 0,-38 23 0,-16 10 0,-11 8 0,11-5 0,-4 3 0,-3 2 0,4-5 0,-3 2 0,0 0 0,3-2 0,-8 7 0,4-2 0,5-4 0,-7 1 0,11-7 0,7-4 0,54-30 0,5-5 0,4-9 0,4-12 0,22-23 0,-6 4 0,11 1 0,-13 8 0,-4 15 0,-7 0 0,-5 6 0,-8 6 0,5-6 0,0 0 0,4-1 0,2 1 0,3-2 0,-4 5 0,2-2 0,-10 14 0,-5 2 0,-1 5 0,-3 3 0,4-3 0,-32 59 0,5-11 0,-17 34 0,10-20 0,9-20 0,5 3 0,-5-9 0,15-15 0,-2-6 0,10-12 0,0-3 0,-1 22 0,1-16 0,-1 16 0,10-24 0,14 0 0,24-5 0,28 2 0,-12-1 0,4 1 0,-10 5 0,0 1 0,3-1 0,-2 0 0,29 14 0,-49-8 0,3-2 0,-24 0 0,-4 5 0,5 4 0,-6-2 0,-3-6 0,-5-7 0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink37.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-08-29T14:41:28.607"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1264 0 24575,'-21'9'0,"-47"41"0,9-4 0,-7 7 0,16-11 0,-3 2 0,-1 1-735,-12 5 0,-4 2 0,2 0 735,2 0 0,1 1 0,1-1 0,6-2 0,1 0 0,2-2 0,-14 10 0,7-3 353,16-6 1,11-9-354,17-23 364,8-8-364,6-18 0,-1-7 0,2-18 1134,-4-25-1134,3-6 0,-2-7 0,3 25 0,1 6 0,2 26 0,0 1 0,0 15 0,0 12 0,-10 54 0,-5 11 0,2 11 0,2-32 0,11-41 0,4-5 0,3 1 0,12 5 0,14 6 0,19-5 0,19 11 0,10-12 0,-27-3 0,-11-10 0,-33-5 0,-6 1 0,-2 3 0,-2-1 0,0 0 0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink38.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-08-29T14:41:30.257"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 177 24575,'4'13'0,"4"-4"0,20 2 0,-6-8 0,10-1 0,-7-6 0,-9 1 0,6-6 0,-13 3 0,13-18 0,-9-3 0,6 0 0,-11 5 0,-8 20 0,-2 0 0,-5 2 0,-9-2 0,-11-1 0,2 0 0,0-1 0,16 3 0,5 1 0,-3 3 0,-8 8 0,4-4 0,-11 14 0,15-16 0,0 12 0,13-6 0,27 30 0,0-12 0,48 24 0,-16-34 0,-4-1 0,-10-15 0,-41-1 0,6-2 0,-12 2 0,6-9 0,-4 5 0,1-5 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="550">623 1 24575,'-15'30'0,"-14"17"0,-4 10 0,2 8 0,-1 1 0,-5 1 0,1 0 0,12-5 0,7-8 0,7-21 0,5-6 0,0-21 0,-14-9 0,6-9 0,-5 7 0,12-3 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1052">373 199 22356,'7'-4'0,"12"1"1077,2 4-1077,24 9 0,-11 10 374,36 40-374,-38-24 0,15 14 0,-39-39 0,-3-9 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1900">738 271 24575,'28'-5'0,"20"-4"0,3-2 0,1-2 0,-25 0 0,-10-6 0,-5-1 0,14-38 0,-12 19 0,3-8 0,-19 30 0,-5 15 0,-5 2 0,2 2 0,1-1 0,-3 5 0,6-5 0,-4 4 0,5 4 0,-9 9 0,0 13 0,-1-3 0,8 5 0,16-10 0,18-2 0,4-5 0,5-6 0,-1-6 0,-14-4 0,13-8 0,-17-4 0,5 1 0,-12 2 0,-12 7 0,3 2 0,-7 0 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2900">521 678 24575,'20'4'0,"0"13"0,1 33 0,-14 15 0,-6 8 0,-5-10 0,-3 4 0,3 8 0,0 8 0,-2-12 0,-8 20 0,10-33 0,1-15 0,1-39 0,-14-26 0,-12-17 0,0 1 0,-4-4 0,22 25 0,3 8 0,26 14 0,-5-4 0,12 6 0,-3-9 0,4-14 0,14-9 0,1-21 0,-6-3 0,-1-5 0,15-33 0,-22 28 0,-3 5 0,-5 12 0,-15 17 0,-5 30 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3667">757 1493 24575,'5'25'0,"10"16"0,0-8 0,2-1 0,5-12 0,-7-18 0,2-1 0,-3-4 0,-3-6 0,1-8 0,1-6 0,-2-13 0,-5 5 0,-14-12 0,-11 16 0,1 5 0,1 13 0,-5 9 0,14 0 0,-10 4 0,16 5 0,2-3 0,0 2 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4550">1098 1358 17431,'19'7'0,"4"47"3190,-3-8-3190,3 30 1225,-12-31-1225,0-23 646,2-15-646,-10-10 2083,18-28-2083,-7-3 0,11-19 0,-13 16 0,-3 16 0,-6 19 0,1 5 0,12 5 0,2-5 0,8-2 0,-1-9 0,23-22 0,-10-1 0,-4-10 0,-2-5 0,-1-19 0,-4-17 0,-29 9 0,0 54 0,1-9 0,5 48 0,11 22 0,1 25 0,-5-16 0,0-1 0,-10-39 0,0-8 0,1 1 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4950">1517 1309 24575,'11'-5'0,"0"2"0,21-12 0,8-14 0,3 5 0,-2-13 0,-14 17 0,-10 7 0,-3 4 0,-10 9 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="7000">2466 1234 24575,'4'-3'0,"18"-1"0,-2 0 0,19 1 0,4-10 0,-4 5 0,14-16 0,-15 7 0,11-10 0,-16 12 0,-4 1 0,-13 6 0,-10 7 0,1-3 0,-9 2 0,-4 1 0,-9-3 0,-20-5 0,5-6 0,-28-27 0,22 0 0,2 2 0,16 17 0,14 21 0,-5 4 0,6-3 0,-1 4 0,8-2 0,22 6 0,24 2 0,23 3 0,-9-5 0,-1 1 0,-34-3 0,-3-1 0,-12 0 0,-10-2 0,-2 0 0,-27 44 0,-11 19 0,-5 11 0,3-6 0,-3 7 0,7-14 0,-5 9 0,1-1 0,6-7 0,-2 8 0,4-6 0,-7 8 0,7-13 0,18-29 0,12-33 0,0-1 0,0 0 0,0 4 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="8817">2872 652 24575,'24'0'0,"14"-2"0,15-1 0,-2-1 0,5-2 0,2-9 0,3-2 0,10 4 0,11-4 0,5-7 0,14-8 0,3-1 0,-14 4-1160,-22 9 1,-8 2 0,7-2 1159,19-6 0,11-3 0,-4 1 0,-21 5 810,6-5-810,-34 14 0,-42 10 0,-26 6 0,2-2 0,-56-6 2668,23 2-2668,-23-5 0,28 6 0,22 1 0,11 2 0,6 0 0,11 0 0,5 2 0,21 6 0,48 10 0,17-1 0,-1-1 0,-6-10 0,-53-6 0,5 0 0,-21 11 0,-9 60 0,-25 8 0,-17 16-476,5-28 0,-9 9 1,-4 4-1,0 0 1,5-6 475,4-1 0,3-4 0,0 0 0,-4 0 0,-13 11 0,-7 3 0,3-6 0,15-15 0,5 14 0,23-64 0,0-9 0,-3-10 0,16-18 0,-8 16 0,19-13 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="9517">5219 154 24575,'-4'-1'0,"-14"27"0,1 30 0,0 9 0,-9 24 0,10-8 0,8-4 0,22-24 0,4-28 0,34-67 0,-13-35 0,-10 11 0,-2-1 0,-5-17 0,-14-6 0,-40 55 0,10 18 0,-11 2 0,3 48 0,15-16 0,-11 23 0,21-31 0,3-10 0,10-15 0,-6 9 0,5-6 0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink39.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-08-29T16:01:25.411"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 376 24575,'24'-3'0,"22"3"0,3 0 0,9 1 0,26 1 0,6 1 0,-25 0 0,3 1 0,1 1-316,7 0 1,2 1 0,-3 0 315,15 0 0,-6 1 116,-15-1 0,-4 0-116,-1-4 0,-6-1 0,10-1 0,5-2 0,-44-1 0,-6 0 714,19 1-714,-15 2 0,25 0 0,-30 0 0,9 0 0,-3-2 0,-7 0 0,-9-1 0,-13-3 0,-15 0 0,-27-42 0,-21-27 0,26 27 0,0 0 0,3 1 0,2 4 0,-10-6 0,14 23 0,9 20 0,7 1 0,0 5 0,6-2 0,0 0 0,1-4 0,6 5 0,5 2 0,24 4 0,14 14 0,11-1 0,21 36 0,-4-2 0,-10 1 0,-8-13 0,-21-20 0,-3 1 0,12 15 0,-11-8 0,-7-1 0,-11-14 0,-8-13 0,-4 4 0,0-3 0,-4 3 0,-3 0 0,-13 19 0,-3 4 0,-10 15 0,-6 13 0,-1 4 0,-5 2 0,4 0 0,1-3 0,6-8 0,6-9 0,8-10 0,8-6 0,6-14 0,1 1 0,1-6 0,2-10 0,2 3 0,2-5 0,4 0 0,0 3 0,4-5 0,-5 7 0,-1-5 0,0 4 0,1-15 0,-2 1 0,9-8 0,-5 2 0,6-4 0,5-8 0,1-17 0,1 11 0,0-21 0,-5 3 0,4-13 0,-4 13 0,-5 17 0,-3 21 0,-4 12 0,-1 0 0,0 4 0,-4-5 0,2 4 0,-4-2 0,3 7 0,-1 0 0,2 2 0</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -9144,7 +9881,7 @@
       <c r="D50" t="s">
         <v>641</v>
       </c>
-      <c r="E50" s="119" t="s">
+      <c r="E50" s="95" t="s">
         <v>739</v>
       </c>
     </row>
@@ -9152,19 +9889,19 @@
       <c r="D51" t="s">
         <v>736</v>
       </c>
-      <c r="E51" s="119"/>
+      <c r="E51" s="95"/>
     </row>
     <row r="52" spans="3:9" x14ac:dyDescent="0.2">
       <c r="D52" t="s">
         <v>737</v>
       </c>
-      <c r="E52" s="119"/>
+      <c r="E52" s="95"/>
     </row>
     <row r="53" spans="3:9" x14ac:dyDescent="0.2">
       <c r="D53" t="s">
         <v>738</v>
       </c>
-      <c r="E53" s="119"/>
+      <c r="E53" s="95"/>
     </row>
     <row r="56" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C56" t="s">
@@ -9349,25 +10086,25 @@
       </c>
     </row>
     <row r="69" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C69" s="120">
+      <c r="C69" s="94">
         <v>1</v>
       </c>
-      <c r="D69" s="120" t="s">
+      <c r="D69" s="94" t="s">
         <v>611</v>
       </c>
-      <c r="E69" s="120">
+      <c r="E69" s="94">
         <v>1</v>
       </c>
-      <c r="F69" s="120">
+      <c r="F69" s="94">
         <v>2</v>
       </c>
-      <c r="G69" s="120" t="s">
+      <c r="G69" s="94" t="s">
         <v>645</v>
       </c>
-      <c r="H69" s="120">
+      <c r="H69" s="94">
         <v>1</v>
       </c>
-      <c r="J69" s="120" t="s">
+      <c r="J69" s="94" t="s">
         <v>744</v>
       </c>
       <c r="K69">
@@ -9375,25 +10112,25 @@
       </c>
     </row>
     <row r="70" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C70" s="120">
+      <c r="C70" s="94">
         <v>1</v>
       </c>
-      <c r="D70" s="120" t="s">
+      <c r="D70" s="94" t="s">
         <v>611</v>
       </c>
-      <c r="E70" s="120">
+      <c r="E70" s="94">
         <v>1</v>
       </c>
-      <c r="F70" s="120">
+      <c r="F70" s="94">
         <v>3</v>
       </c>
-      <c r="G70" s="120" t="s">
+      <c r="G70" s="94" t="s">
         <v>646</v>
       </c>
-      <c r="H70" s="120">
+      <c r="H70" s="94">
         <v>1</v>
       </c>
-      <c r="J70" s="120" t="s">
+      <c r="J70" s="94" t="s">
         <v>745</v>
       </c>
       <c r="K70">
@@ -9453,25 +10190,25 @@
       </c>
     </row>
     <row r="73" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C73" s="120">
+      <c r="C73" s="94">
         <v>2</v>
       </c>
-      <c r="D73" s="120" t="s">
+      <c r="D73" s="94" t="s">
         <v>645</v>
       </c>
-      <c r="E73" s="120">
+      <c r="E73" s="94">
         <v>1</v>
       </c>
-      <c r="F73" s="120">
+      <c r="F73" s="94">
         <v>3</v>
       </c>
-      <c r="G73" s="120" t="s">
+      <c r="G73" s="94" t="s">
         <v>646</v>
       </c>
-      <c r="H73" s="120">
+      <c r="H73" s="94">
         <v>1</v>
       </c>
-      <c r="J73" s="120" t="s">
+      <c r="J73" s="94" t="s">
         <v>748</v>
       </c>
       <c r="K73">
@@ -9583,25 +10320,25 @@
       </c>
     </row>
     <row r="78" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C78" s="120">
+      <c r="C78" s="94">
         <v>4</v>
       </c>
-      <c r="D78" s="120" t="s">
+      <c r="D78" s="94" t="s">
         <v>647</v>
       </c>
-      <c r="E78" s="120">
+      <c r="E78" s="94">
         <v>2</v>
       </c>
-      <c r="F78" s="120">
+      <c r="F78" s="94">
         <v>5</v>
       </c>
-      <c r="G78" s="120" t="s">
+      <c r="G78" s="94" t="s">
         <v>648</v>
       </c>
-      <c r="H78" s="120">
+      <c r="H78" s="94">
         <v>2</v>
       </c>
-      <c r="J78" s="120" t="s">
+      <c r="J78" s="94" t="s">
         <v>753</v>
       </c>
       <c r="K78">
@@ -10429,14 +11166,14 @@
       </c>
     </row>
     <row r="166" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C166" s="119" t="s">
+      <c r="C166" s="95" t="s">
         <v>726</v>
       </c>
-      <c r="D166" s="119"/>
-      <c r="G166" s="119" t="s">
+      <c r="D166" s="95"/>
+      <c r="G166" s="95" t="s">
         <v>588</v>
       </c>
-      <c r="H166" s="119"/>
+      <c r="H166" s="95"/>
     </row>
     <row r="167" spans="3:8" x14ac:dyDescent="0.2">
       <c r="C167" s="1">
@@ -10586,6 +11323,418 @@
     <mergeCell ref="E50:E53"/>
     <mergeCell ref="C166:D166"/>
     <mergeCell ref="G166:H166"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C17B837-974D-B54B-ABEA-DED5637FC833}">
+  <dimension ref="B6:M87"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="12:13" x14ac:dyDescent="0.2">
+      <c r="L6" t="s">
+        <v>94</v>
+      </c>
+      <c r="M6" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="7" spans="12:13" x14ac:dyDescent="0.2">
+      <c r="L7" t="s">
+        <v>308</v>
+      </c>
+      <c r="M7" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="13" spans="12:13" x14ac:dyDescent="0.2">
+      <c r="L13" t="s">
+        <v>561</v>
+      </c>
+      <c r="M13" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="14" spans="12:13" x14ac:dyDescent="0.2">
+      <c r="L14" t="s">
+        <v>562</v>
+      </c>
+      <c r="M14" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="26" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K26" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="27" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K27" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="28" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K28" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="29" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K29" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="30" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K30" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="C37" t="s">
+        <v>284</v>
+      </c>
+      <c r="E37" t="s">
+        <v>780</v>
+      </c>
+      <c r="G37" s="111" t="s">
+        <v>781</v>
+      </c>
+      <c r="H37" s="111"/>
+      <c r="I37" s="111"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="C38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
+    </row>
+    <row r="49" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="E49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1"/>
+    </row>
+    <row r="50" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+    </row>
+    <row r="51" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="C52" s="121" t="s">
+        <v>782</v>
+      </c>
+      <c r="E52" s="121" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="53" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="C53" s="122"/>
+      <c r="E53" s="122"/>
+    </row>
+    <row r="54" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="C54" s="122"/>
+      <c r="E54" s="122"/>
+    </row>
+    <row r="55" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C55" s="123"/>
+      <c r="E55" s="123"/>
+    </row>
+    <row r="63" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B63" s="1"/>
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="J63" s="1"/>
+      <c r="K63" s="1"/>
+      <c r="L63" s="1"/>
+    </row>
+    <row r="64" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="J64" s="1"/>
+      <c r="K64" s="1"/>
+      <c r="L64" s="1"/>
+    </row>
+    <row r="65" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B65" s="1"/>
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+      <c r="J65" s="1"/>
+      <c r="K65" s="1"/>
+      <c r="L65" s="1"/>
+    </row>
+    <row r="66" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+      <c r="J66" s="1"/>
+      <c r="K66" s="1"/>
+      <c r="L66" s="1"/>
+    </row>
+    <row r="67" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B67" s="1"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1"/>
+      <c r="J67" s="1"/>
+      <c r="K67" s="1"/>
+      <c r="L67" s="1"/>
+    </row>
+    <row r="68" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+      <c r="J68" s="1"/>
+      <c r="K68" s="1"/>
+      <c r="L68" s="1"/>
+    </row>
+    <row r="69" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B69" s="1"/>
+      <c r="C69" s="1"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+      <c r="J69" s="1"/>
+      <c r="K69" s="1"/>
+      <c r="L69" s="1"/>
+    </row>
+    <row r="70" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="J70" s="1"/>
+      <c r="K70" s="1"/>
+      <c r="L70" s="1"/>
+    </row>
+    <row r="71" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="J71" s="1"/>
+      <c r="K71" s="1"/>
+      <c r="L71" s="1"/>
+    </row>
+    <row r="72" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B72" s="1"/>
+      <c r="C72" s="1"/>
+      <c r="D72" s="1"/>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="1"/>
+      <c r="H72" s="1"/>
+      <c r="J72" s="1"/>
+      <c r="K72" s="1"/>
+      <c r="L72" s="1"/>
+    </row>
+    <row r="73" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B73" s="1"/>
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1"/>
+      <c r="G73" s="1"/>
+      <c r="H73" s="1"/>
+      <c r="J73" s="1"/>
+      <c r="K73" s="1"/>
+      <c r="L73" s="1"/>
+    </row>
+    <row r="74" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="1"/>
+      <c r="F74" s="1"/>
+      <c r="G74" s="1"/>
+      <c r="H74" s="1"/>
+      <c r="J74" s="1"/>
+      <c r="K74" s="1"/>
+      <c r="L74" s="1"/>
+    </row>
+    <row r="75" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B75" s="1"/>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
+    </row>
+    <row r="76" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B76" s="1"/>
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+      <c r="H76" s="1"/>
+    </row>
+    <row r="77" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B77" s="1"/>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+      <c r="H77" s="1"/>
+    </row>
+    <row r="84" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B84" t="s">
+        <v>284</v>
+      </c>
+      <c r="D84" t="s">
+        <v>780</v>
+      </c>
+      <c r="F84" s="111" t="s">
+        <v>781</v>
+      </c>
+      <c r="G84" s="111"/>
+      <c r="H84" s="111"/>
+    </row>
+    <row r="85" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B85" t="s">
+        <v>274</v>
+      </c>
+      <c r="D85" t="s">
+        <v>548</v>
+      </c>
+      <c r="E85" s="95" t="s">
+        <v>784</v>
+      </c>
+      <c r="G85" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="86" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B86" t="s">
+        <v>548</v>
+      </c>
+      <c r="D86" t="s">
+        <v>582</v>
+      </c>
+      <c r="E86" s="95"/>
+      <c r="G86" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="87" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B87" t="s">
+        <v>582</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="C52:C55"/>
+    <mergeCell ref="E52:E55"/>
+    <mergeCell ref="F84:H84"/>
+    <mergeCell ref="E85:E86"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -13172,7 +14321,7 @@
       </c>
       <c r="J56" t="str">
         <f ca="1">TEXT(NOW(),"YYYY-MM-DD")</f>
-        <v>2026-08-23</v>
+        <v>2026-08-29</v>
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.2">
@@ -13181,7 +14330,7 @@
       </c>
       <c r="J57" t="str">
         <f ca="1">TEXT(NOW(),"dddd, mmm DD yyyy")</f>
-        <v>Sunday, Aug 23 2026</v>
+        <v>Saturday, Aug 29 2026</v>
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.2">
@@ -15897,17 +17046,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="111" t="s">
         <v>585</v>
       </c>
-      <c r="C2" s="109"/>
-      <c r="D2" s="109"/>
-      <c r="E2" s="109"/>
-      <c r="G2" s="109" t="s">
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="G2" s="111" t="s">
         <v>586</v>
       </c>
-      <c r="H2" s="109"/>
-      <c r="I2" s="109"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="41"/>
@@ -16041,12 +17190,12 @@
       <c r="F20" s="52"/>
       <c r="G20" s="53"/>
       <c r="H20" s="54"/>
-      <c r="J20" s="110" t="s">
+      <c r="J20" s="112" t="s">
         <v>587</v>
       </c>
-      <c r="K20" s="111"/>
-      <c r="L20" s="111"/>
-      <c r="M20" s="112"/>
+      <c r="K20" s="113"/>
+      <c r="L20" s="113"/>
+      <c r="M20" s="114"/>
       <c r="O20" t="s">
         <v>590</v>
       </c>
@@ -16059,10 +17208,10 @@
       <c r="F21" s="52"/>
       <c r="G21" s="53"/>
       <c r="H21" s="54"/>
-      <c r="J21" s="113"/>
-      <c r="K21" s="114"/>
-      <c r="L21" s="114"/>
-      <c r="M21" s="115"/>
+      <c r="J21" s="115"/>
+      <c r="K21" s="116"/>
+      <c r="L21" s="116"/>
+      <c r="M21" s="117"/>
       <c r="P21" t="s">
         <v>592</v>
       </c>
@@ -16075,10 +17224,10 @@
       <c r="F22" s="52"/>
       <c r="G22" s="53"/>
       <c r="H22" s="54"/>
-      <c r="J22" s="113"/>
-      <c r="K22" s="114"/>
-      <c r="L22" s="114"/>
-      <c r="M22" s="115"/>
+      <c r="J22" s="115"/>
+      <c r="K22" s="116"/>
+      <c r="L22" s="116"/>
+      <c r="M22" s="117"/>
       <c r="Q22" t="s">
         <v>594</v>
       </c>
@@ -16091,10 +17240,10 @@
       <c r="F23" s="52"/>
       <c r="G23" s="53"/>
       <c r="H23" s="54"/>
-      <c r="J23" s="116"/>
-      <c r="K23" s="117"/>
-      <c r="L23" s="117"/>
-      <c r="M23" s="118"/>
+      <c r="J23" s="118"/>
+      <c r="K23" s="119"/>
+      <c r="L23" s="119"/>
+      <c r="M23" s="120"/>
       <c r="P23" t="s">
         <v>593</v>
       </c>
@@ -16107,12 +17256,12 @@
       <c r="F24" s="52"/>
       <c r="G24" s="53"/>
       <c r="H24" s="54"/>
-      <c r="J24" s="94" t="s">
+      <c r="J24" s="96" t="s">
         <v>589</v>
       </c>
-      <c r="K24" s="95"/>
-      <c r="L24" s="95"/>
-      <c r="M24" s="96"/>
+      <c r="K24" s="97"/>
+      <c r="L24" s="97"/>
+      <c r="M24" s="98"/>
       <c r="O24" t="s">
         <v>591</v>
       </c>
@@ -16125,28 +17274,28 @@
       <c r="F25" s="52"/>
       <c r="G25" s="53"/>
       <c r="H25" s="54"/>
-      <c r="J25" s="97"/>
-      <c r="K25" s="98"/>
-      <c r="L25" s="98"/>
-      <c r="M25" s="99"/>
+      <c r="J25" s="99"/>
+      <c r="K25" s="100"/>
+      <c r="L25" s="100"/>
+      <c r="M25" s="101"/>
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.2">
       <c r="F26" s="52"/>
       <c r="G26" s="53"/>
       <c r="H26" s="54"/>
-      <c r="J26" s="97"/>
-      <c r="K26" s="98"/>
-      <c r="L26" s="98"/>
-      <c r="M26" s="99"/>
+      <c r="J26" s="99"/>
+      <c r="K26" s="100"/>
+      <c r="L26" s="100"/>
+      <c r="M26" s="101"/>
     </row>
     <row r="27" spans="2:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="F27" s="52"/>
       <c r="G27" s="53"/>
       <c r="H27" s="54"/>
-      <c r="J27" s="100"/>
-      <c r="K27" s="101"/>
-      <c r="L27" s="101"/>
-      <c r="M27" s="102"/>
+      <c r="J27" s="102"/>
+      <c r="K27" s="103"/>
+      <c r="L27" s="103"/>
+      <c r="M27" s="104"/>
       <c r="O27" t="s">
         <v>595</v>
       </c>
@@ -16188,22 +17337,22 @@
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="45"/>
-      <c r="J35" s="110" t="s">
+      <c r="J35" s="112" t="s">
         <v>588</v>
       </c>
-      <c r="K35" s="111"/>
-      <c r="L35" s="111"/>
-      <c r="M35" s="112"/>
+      <c r="K35" s="113"/>
+      <c r="L35" s="113"/>
+      <c r="M35" s="114"/>
     </row>
     <row r="36" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B36" s="44"/>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="45"/>
-      <c r="J36" s="113"/>
-      <c r="K36" s="114"/>
-      <c r="L36" s="114"/>
-      <c r="M36" s="115"/>
+      <c r="J36" s="115"/>
+      <c r="K36" s="116"/>
+      <c r="L36" s="116"/>
+      <c r="M36" s="117"/>
       <c r="O36" t="s">
         <v>598</v>
       </c>
@@ -16216,10 +17365,10 @@
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="45"/>
-      <c r="J37" s="113"/>
-      <c r="K37" s="114"/>
-      <c r="L37" s="114"/>
-      <c r="M37" s="115"/>
+      <c r="J37" s="115"/>
+      <c r="K37" s="116"/>
+      <c r="L37" s="116"/>
+      <c r="M37" s="117"/>
       <c r="O37" t="s">
         <v>599</v>
       </c>
@@ -16232,22 +17381,22 @@
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="45"/>
-      <c r="J38" s="116"/>
-      <c r="K38" s="117"/>
-      <c r="L38" s="117"/>
-      <c r="M38" s="118"/>
+      <c r="J38" s="118"/>
+      <c r="K38" s="119"/>
+      <c r="L38" s="119"/>
+      <c r="M38" s="120"/>
     </row>
     <row r="39" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B39" s="44"/>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
       <c r="E39" s="45"/>
-      <c r="J39" s="94" t="s">
+      <c r="J39" s="96" t="s">
         <v>600</v>
       </c>
-      <c r="K39" s="95"/>
-      <c r="L39" s="95"/>
-      <c r="M39" s="96"/>
+      <c r="K39" s="97"/>
+      <c r="L39" s="97"/>
+      <c r="M39" s="98"/>
       <c r="O39" t="s">
         <v>598</v>
       </c>
@@ -16266,10 +17415,10 @@
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="45"/>
-      <c r="J40" s="97"/>
-      <c r="K40" s="98"/>
-      <c r="L40" s="98"/>
-      <c r="M40" s="99"/>
+      <c r="J40" s="99"/>
+      <c r="K40" s="100"/>
+      <c r="L40" s="100"/>
+      <c r="M40" s="101"/>
       <c r="O40" t="s">
         <v>599</v>
       </c>
@@ -16288,10 +17437,10 @@
       <c r="C41" s="47"/>
       <c r="D41" s="47"/>
       <c r="E41" s="48"/>
-      <c r="J41" s="97"/>
-      <c r="K41" s="98"/>
-      <c r="L41" s="98"/>
-      <c r="M41" s="99"/>
+      <c r="J41" s="99"/>
+      <c r="K41" s="100"/>
+      <c r="L41" s="100"/>
+      <c r="M41" s="101"/>
     </row>
     <row r="42" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B42" s="49" t="s">
@@ -16306,52 +17455,52 @@
       <c r="E42" s="59" t="s">
         <v>602</v>
       </c>
-      <c r="J42" s="100"/>
-      <c r="K42" s="101"/>
-      <c r="L42" s="101"/>
-      <c r="M42" s="102"/>
+      <c r="J42" s="102"/>
+      <c r="K42" s="103"/>
+      <c r="L42" s="103"/>
+      <c r="M42" s="104"/>
     </row>
     <row r="43" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B43" s="52"/>
       <c r="C43" s="53"/>
       <c r="D43" s="54"/>
       <c r="E43" s="60"/>
-      <c r="J43" s="94" t="s">
+      <c r="J43" s="96" t="s">
         <v>601</v>
       </c>
-      <c r="K43" s="95"/>
-      <c r="L43" s="95"/>
-      <c r="M43" s="96"/>
+      <c r="K43" s="97"/>
+      <c r="L43" s="97"/>
+      <c r="M43" s="98"/>
     </row>
     <row r="44" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B44" s="52"/>
       <c r="C44" s="53"/>
       <c r="D44" s="54"/>
       <c r="E44" s="60"/>
-      <c r="J44" s="97"/>
-      <c r="K44" s="98"/>
-      <c r="L44" s="98"/>
-      <c r="M44" s="99"/>
+      <c r="J44" s="99"/>
+      <c r="K44" s="100"/>
+      <c r="L44" s="100"/>
+      <c r="M44" s="101"/>
     </row>
     <row r="45" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B45" s="52"/>
       <c r="C45" s="53"/>
       <c r="D45" s="54"/>
       <c r="E45" s="60"/>
-      <c r="J45" s="97"/>
-      <c r="K45" s="98"/>
-      <c r="L45" s="98"/>
-      <c r="M45" s="99"/>
+      <c r="J45" s="99"/>
+      <c r="K45" s="100"/>
+      <c r="L45" s="100"/>
+      <c r="M45" s="101"/>
     </row>
     <row r="46" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B46" s="52"/>
       <c r="C46" s="53"/>
       <c r="D46" s="54"/>
       <c r="E46" s="60"/>
-      <c r="J46" s="100"/>
-      <c r="K46" s="101"/>
-      <c r="L46" s="101"/>
-      <c r="M46" s="102"/>
+      <c r="J46" s="102"/>
+      <c r="K46" s="103"/>
+      <c r="L46" s="103"/>
+      <c r="M46" s="104"/>
     </row>
     <row r="47" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B47" s="52"/>
@@ -16402,12 +17551,12 @@
     </row>
     <row r="58" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="59" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="E59" s="103" t="s">
+      <c r="E59" s="105" t="s">
         <v>608</v>
       </c>
-      <c r="F59" s="104"/>
-      <c r="G59" s="104"/>
-      <c r="H59" s="105"/>
+      <c r="F59" s="106"/>
+      <c r="G59" s="106"/>
+      <c r="H59" s="107"/>
       <c r="J59" t="s">
         <v>609</v>
       </c>
@@ -16416,10 +17565,10 @@
       <c r="B60" t="s">
         <v>604</v>
       </c>
-      <c r="E60" s="106"/>
-      <c r="F60" s="107"/>
-      <c r="G60" s="107"/>
-      <c r="H60" s="108"/>
+      <c r="E60" s="108"/>
+      <c r="F60" s="109"/>
+      <c r="G60" s="109"/>
+      <c r="H60" s="110"/>
     </row>
     <row r="61" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B61" t="s">

</xml_diff>